<commit_message>
[Codex] refactor: 集中地圖掉落與 R0-R10 配置
</commit_message>
<xml_diff>
--- a/config/Excel/NPC.xlsx
+++ b/config/Excel/NPC.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPC" sheetId="1" r:id="R68ea60a2b86e4c8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPC" sheetId="1" r:id="R59a95684e2c54893"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2237,7 +2237,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra60086d77fe64783"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a3aa16fea8c468e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>